<commit_message>
mejoras de arquitectura logica
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R6057c451c6214cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Re296eeb6affb499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Rb9d7b4183f5a45a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R384a1b08a6174afa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -857,6 +857,32 @@
         <x:v>Parcial: preliminar incorporado; revisión técnica pendiente</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="165" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Integrar la revisión 67 de arquitectura lógica y mejorar claridad y coherencia del subdocumento 4.1.</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Solicitud de Álvaro; arquitectura_logica_version67.md, revisión 67.</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Subdoc 4.1 (arquitectura lógica)</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Se actualizan Markdown y LaTeX: ACL exclusiva del ERP, hub EDI, datos offline, identidad, roles de sitio y observabilidad. Se corrigen autonomía mínima, flujos de acceso y garantías no demostradas. Arquitectura física y Entrega 1 intactas.</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>4.1–4.7; 04_arquitectura/entrega_2/texto/arquitectura_logica.md y latex/subdoc_4.1.tex; README de revisión.</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>Parcial: integración editorial terminada; identidad offline, matriz de roles, DR y concordancia gráfica pendientes de validación.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
realizacion de robustes arc logica, se crearon diagramas nuevos que dictan el recorrido de los datos
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R60e344679bed4999"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rc2bfba8e57f041ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R4ada3191f3054ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rfcd304ad1d3b4081"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -909,6 +909,162 @@
         <x:v>Limpieza editorial completada. La autorización de relevos sin IdP y la concordancia de los diagramas requieren validación técnica.</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="108" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Diagramas del 4.1 ilegibles, repetidos y desconectados de la explicación; falta secuencia del pedido y modelo de dominio.</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Revisión del evaluador, Subdocumento 4.1, pp. 9-10.</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Subdoc 4.1</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Se sustituyen las vistas repetitivas e ilegibles del cuerpo por una vista general legible y cuatro diagramas específicos: pedido con conexión, pedido sin conexión, acceso local y dominio. Los originales se conservan en la biblioteca. Cada figura nueva se cita y analiza en su sección.</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>4.1, Capas 2-5; Modelo de datos conceptual; diagramas ARQL-15 a ARQL-19.</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>Atendida en texto; pendiente revisión visual del PDF compilado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="108" customHeight="1">
+      <x:c r="A18" s="4" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>No se identifican los doce módulos con actor, interfaces y etapa ni se muestra requerimiento a módulo y capa.</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>Revisión del evaluador, Subdocumento 4.1, pp. 9-10.</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>Subdoc 4.1</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Se completa la tabla de M1-M12 con actor y etapa y se agrega trazabilidad RF-módulo-capa con evidencia; se mantiene el detalle exhaustivo como responsabilidad del Formulario T-12.</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>4.1, Módulos funcionales y límites de contexto; Tablas de módulos y trazabilidad lógica.</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>Atendida en 4.1; contrastar contra T-12 consolidado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="108" customHeight="1">
+      <x:c r="A19" s="4" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B19" s="4" t="str">
+        <x:v>Identidad de ocho horas y puerta de enlace remota no explican dos relevos ni el trabajo de 120 terminales durante 24 horas sin nube.</x:v>
+      </x:c>
+      <x:c r="C19" s="4" t="str">
+        <x:v>Revisión del evaluador, Subdocumento 4.1, p. 10; consistencia transversal, p. 17.</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="str">
+        <x:v>Subdoc 4.1</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="str">
+        <x:v>Se define manifiesto firmado renovado cada hora, verificador de turno y puerta de API local con controles de esquema, tasa, autorización y auditoría. La prueba parte antes de dos relevos y reconoce el límite de revocación remota.</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>4.1, Capas 3 y 7; Figura de acceso local; funciones sin conexión.</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>Diseño lógico atendido; prueba de 24 h pendiente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="108" customHeight="1">
+      <x:c r="A20" s="4" t="str">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B20" s="4" t="str">
+        <x:v>No se demuestra aplicación de SOLID, orquestación/coreografía ni cobertura de los cinco ambientes del SDLC.</x:v>
+      </x:c>
+      <x:c r="C20" s="4" t="str">
+        <x:v>Revisión del evaluador, Subdocumento 4.1, pp. 9-10.</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="str">
+        <x:v>Subdoc 4.1</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="str">
+        <x:v>Se sitúan los cinco principios en contratos concretos, se distingue confirmación síncrona de reacción por eventos y se especifica qué se prueba y promueve en Desarrollo, QA, Preproducción, Producción y DR.</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>4.1, Integración y eventos; Ambientes del ciclo de vida; Patrones de diseño.</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str">
+        <x:v>Atendida en diseño; verificar topología con 4.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="108" customHeight="1">
+      <x:c r="A21" s="4" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="str">
+        <x:v>La decisión sobre excursión térmica difiere entre 3 y 4.1; el conductor no debe liberar un lote.</x:v>
+      </x:c>
+      <x:c r="C21" s="4" t="str">
+        <x:v>Revisión del evaluador, Subdocumentos 3 y 4.1, pp. 8 y 10.</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="str">
+        <x:v>Subdoc 4.1</x:v>
+      </x:c>
+      <x:c r="E21" s="4" t="str">
+        <x:v>Se fija retención preventiva automática local en M9/M5 y liberación exclusiva por Calidad, con registro de umbral, lote, causa y autoridad. El conductor solo informa y conserva la carga.</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>4.1, M9 Calidad; Integración y eventos; Reglas de reconciliación.</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="str">
+        <x:v>4.1 atendido; falta armonizar Subdoc 3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="108" customHeight="1">
+      <x:c r="A22" s="4" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B22" s="4" t="str">
+        <x:v>La comparación de alternativas es superficial y remite a un ADR alojado en 4.2 que incluye precios.</x:v>
+      </x:c>
+      <x:c r="C22" s="4" t="str">
+        <x:v>Revisión del evaluador, Subdocumento 4.1, p. 10; observación 4.2, p. 13.</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="str">
+        <x:v>Subdoc 4.1</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="str">
+        <x:v>Se hace autocontenido el registro lógico con alternativa, criterio y consecuencia de siete decisiones, y se eliminan las referencias a un adjunto inexistente. Las elecciones tecnológicas se explican por su función en Puelche.</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="str">
+        <x:v>4.1, Tecnologías seleccionadas; Registro de decisiones; Comparación de alternativas.</x:v>
+      </x:c>
+      <x:c r="G22" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H22" s="4" t="str">
+        <x:v>Atendida en 4.1; revisión humana pendiente</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
cambio de framework: laravel
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R4ada3191f3054ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rfcd304ad1d3b4081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R9666066b2813431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rb614f52b84e34385"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1065,6 +1065,32 @@
         <x:v>Atendida en 4.1; revisión humana pendiente</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="108" customHeight="1">
+      <x:c r="A23" s="4" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B23" s="4" t="str">
+        <x:v>La elección de Django para el backend ya no representa la plataforma acordada para la arquitectura lógica; se requiere conservar contratos, datos y operación offline al adoptar Laravel.</x:v>
+      </x:c>
+      <x:c r="C23" s="4" t="str">
+        <x:v>Solicitud de Álvaro, 25-09-2026; contraste de 4.1 con la rama Guillermo-subdoc4-consistencia.</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="str">
+        <x:v>Subdoc 4.1 (arquitectura lógica)</x:v>
+      </x:c>
+      <x:c r="E23" s="4" t="str">
+        <x:v>Se define Laravel 13/PHP 8.5 en M1--M12, límites PSR-4, persistencia PostGIS, Keycloak OIDC, consumidor JSON de SQS separado de trabajos Laravel, adaptador RabbitMQ, pruebas y transición por sitio con escritor único y reversión.</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="str">
+        <x:v>4.1.1 Tecnologías; Capa 4; Capa 5; Capa 7; Detalle de tecnologías; Implantación progresiva; ADR-01/05/12; Alternativas.</x:v>
+      </x:c>
+      <x:c r="G23" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H23" s="4" t="str">
+        <x:v>Atendida en 4.1; 4.2, T-11 y ADR físicos pendientes de armonización</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
actualizacion de coherencia: diagrama de arquitectura logica
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R9666066b2813431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rb614f52b84e34385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Rc4877283625f4917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rb8f08f3eb8e1460e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +49,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyAlignment="1">
@@ -60,6 +60,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1091,6 +1094,110 @@
         <x:v>Atendida en 4.1; 4.2, T-11 y ADR físicos pendientes de armonización</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="108" customHeight="1">
+      <x:c r="A24" s="4" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B24" s="4" t="str">
+        <x:v>Las tablas extensas del Subdocumento 4.1 se parten entre páginas o desplazan el análisis del cuerpo principal.</x:v>
+      </x:c>
+      <x:c r="C24" s="4" t="str">
+        <x:v>Bases/aclaraciones-licitacion.md, sección 5; revisión de paginación de 4.1.</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>Subdoc 4.1 (arquitectura lógica)</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>Se trasladan doce catálogos y matrices extensas a los anexos 4.1-A a 4.1-L. El cuerpo conserva síntesis, análisis y citas expresas al anexo correspondiente.</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="str">
+        <x:v>4.1, eventos, gobierno, carga masiva, módulos, trazabilidad, límites de contexto, interfaces, volumen, continuidad offline, reconciliación y decisiones del caso; anexos 4.1-A a 4.1-L.</x:v>
+      </x:c>
+      <x:c r="G24" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H24" s="4" t="str">
+        <x:v>Atendida en 4.1; compilación y revisión visual pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="108" customHeight="1">
+      <x:c r="A25" s="4" t="str">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>La vista general de arquitectura lógica aún mostraba el stack anterior y el archivo de anexos no encontraba la plantilla al abrirse desde su carpeta.</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>Revisión del Subdocumento 4.1 y solicitud de Álvaro, 26-09-2026.</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>Subdoc 4.1 (arquitectura lógica)</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>Se corrigió la ruta de la clase y la portada del archivo de anexos; se compiló su PDF. Se recreó el diagrama general con Laravel/PHP, se actualizó la figura resumida del 4.1 y se verificó su legibilidad impresa.</x:v>
+      </x:c>
+      <x:c r="F25" s="4" t="str">
+        <x:v>4.1, Figura 4.1; Diagramas/arquitectura_logica_actual/ARQL-19 y ARQL-20; anexos_4.1.tex y anexos_4.1.pdf.</x:v>
+      </x:c>
+      <x:c r="G25" s="4" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H25" s="4" t="str">
+        <x:v>Atendida en 4.1; revisión humana del consolidado pendiente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="108" customHeight="1">
+      <x:c r="A26" t="str">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>Integrar las vistas Laravel y descripciones elaboradas en paralelo, preservando los cambios locales del 4.1.</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Solicitud de Álvaro; aporte de Tomás, commit b08b623.</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Subdoc 4.1: diagramas y vistas por actor</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>Se integraron 14 PNG, TXT y capa de negocio. Se precisaron las descripciones del conductor externo y de TI; se documentaron diferencias de TTL, acceso HHT y etiqueta residual antes de sustituir figuras consolidadas.</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>Diagramas/arquitectura_logica_actual/cambios laravel/LECTURA_DIAGRAMAS.md y capas/04_negocio.png.</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Integrado; armonización visual y revisión humana pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="108" customHeight="1">
+      <x:c r="A27" t="str">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Explicitar el aporte de la arquitectura lógica a la continuidad del negocio y de las TIC.</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Bases Técnicas Transversales RT-10.03/04; ISO 22301:2019 e ISO/IEC 27031:2025.</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Subdoc 4.1: patrones de diseño y continuidad</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>Se incorporó el vínculo entre normas, funciones offline, dependencias, recuperación y reconciliación. Se definieron pruebas y la remisión al Subdoc 11 para BIA, activación y procedimientos; no se afirma certificación.</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>4.1, Patrones de diseño y continuidad; Referencias. https://www.iso.org/standard/75106.html ; https://www.iso.org/standard/27031</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Diseño documentado; pruebas y revisión humana pendientes</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
tengo sueño y debo dormir 3:00
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Rc4877283625f4917"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rb8f08f3eb8e1460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Raec8ab711cc3469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rad8b71f4dba64ee9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1198,6 +1198,32 @@
         <x:v>Diseño documentado; pruebas y revisión humana pendientes</x:v>
       </x:c>
     </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Presentar primero la vista general completa y después la síntesis de la arquitectura lógica.</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Solicitud de Álvaro, 27-09-2026.</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Subdoc 4.1: capas de arquitectura</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Se incorporó ARQL-01 de Tomás como primera figura y se mantuvo ARQL-19 a continuación, en páginas independientes, con referencias y pies actualizados.</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>4.1, Figuras 4.1 y 4.2.</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Implementado; revisión humana del consolidado pendiente</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
mejora subdoc 4.1: diagramas
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Raec8ab711cc3469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rad8b71f4dba64ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R006e3f86ee334562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R1cb70db3a6464251"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1203,16 +1203,16 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>Presentar primero la vista general completa y después la síntesis de la arquitectura lógica.</x:v>
+        <x:v>Presentar primero la vista general completa y después la síntesis, con una descripción propia para cada diagrama.</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>Solicitud de Álvaro, 27-09-2026.</x:v>
+        <x:v>Solicitudes de Álvaro, 27 y 28-09-2026.</x:v>
       </x:c>
       <x:c r="D28" t="str">
         <x:v>Subdoc 4.1: capas de arquitectura</x:v>
       </x:c>
       <x:c r="E28" t="str">
-        <x:v>Se incorporó ARQL-01 de Tomás como primera figura y se mantuvo ARQL-19 a continuación, en páginas independientes, con referencias y pies actualizados.</x:v>
+        <x:v>Se incorporó ARQL-01 de Tomás antes de ARQL-19. Cada figura incluye su descripción y guía de lectura; se ajustó el tamaño de la síntesis para compartir página con su explicación.</x:v>
       </x:c>
       <x:c r="F28" t="str">
         <x:v>4.1, Figuras 4.1 y 4.2.</x:v>

</xml_diff>

<commit_message>
reorganizacion de carpetas para ser subido a drive
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R006e3f86ee334562"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R1cb70db3a6464251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R406c256d1ac347b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R4650b984a0c44c78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1224,6 +1224,162 @@
         <x:v>Implementado; revisión humana del consolidado pendiente</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="150" customHeight="1">
+      <x:c r="A29" s="3" t="str">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B29" s="3" t="str">
+        <x:v>Unificar las fuentes lógicas Laravel y corregir contradicciones de continuidad.</x:v>
+      </x:c>
+      <x:c r="C29" s="3" t="str">
+        <x:v>Auditoría comunicada por Álvaro, 29-09-2026; Aclaraciones §§3 y 7.1.</x:v>
+      </x:c>
+      <x:c r="D29" s="3" t="str">
+        <x:v>4.1 y Markdown lógico</x:v>
+      </x:c>
+      <x:c r="E29" s="3" t="str">
+        <x:v>Se sincronizan tecnologías, exposición, separación OpenAS2/M11 y CDC exclusivo de Talca. No se modifica 4.2.</x:v>
+      </x:c>
+      <x:c r="F29" s="3" t="str">
+        <x:v>Capas 2, 4, 6, 7; catálogo; texto lógico.</x:v>
+      </x:c>
+      <x:c r="G29" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H29" s="3" t="str">
+        <x:v>Implementado en lógica; coherencia integrada requiere consolidar 4.2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="150" customHeight="1">
+      <x:c r="A30" s="3" t="str">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B30" s="3" t="str">
+        <x:v>Resolver despacho de 96 camiones ante falla ERP/DTE.</x:v>
+      </x:c>
+      <x:c r="C30" s="3" t="str">
+        <x:v>Caso 02, ventana 05:30–07:00; observación prioritaria 2.</x:v>
+      </x:c>
+      <x:c r="D30" s="3" t="str">
+        <x:v>4.1 POD–DTE–acuse</x:v>
+      </x:c>
+      <x:c r="E30" s="3" t="str">
+        <x:v>Se definen estados, consulta idempotente y control de liberación. AL-DTE-01 exige procedimiento del CLIENTE y ensayo de 96 salidas.</x:v>
+      </x:c>
+      <x:c r="F30" s="3" t="str">
+        <x:v>4.1 control de liberación; Anexo M, AL-DTE-01.</x:v>
+      </x:c>
+      <x:c r="G30" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H30" s="3" t="str">
+        <x:v>Diseño y protocolo definidos; aprobación tributaria y ensayo no acreditados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="150" customHeight="1">
+      <x:c r="A31" s="3" t="str">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B31" s="3" t="str">
+        <x:v>Demostrar RPO15 con pérdida de sitio y WAN; probar autonomía con dos relevos.</x:v>
+      </x:c>
+      <x:c r="C31" s="3" t="str">
+        <x:v>RT-07.04; RT-03.10/13; observaciones 3 y 5.</x:v>
+      </x:c>
+      <x:c r="D31" s="3" t="str">
+        <x:v>4.1 continuidad y funciones offline</x:v>
+      </x:c>
+      <x:c r="E31" s="3" t="str">
+        <x:v>Se retira garantía incondicional sin sustento. AL-DR-01 y AL-OFF-01 definen medición y aceptación; AL-BR-01 registra brecha.</x:v>
+      </x:c>
+      <x:c r="F31" s="3" t="str">
+        <x:v>Anexo M; reconciliación y condiciones de diseño.</x:v>
+      </x:c>
+      <x:c r="G31" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H31" s="3" t="str">
+        <x:v>Pruebas no ejecutadas. Protección externa bajo aislamiento no resuelta.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="150" customHeight="1">
+      <x:c r="A32" s="3" t="str">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B32" s="3" t="str">
+        <x:v>Completar modo, volumen, disponibilidad y conducta de cada integración.</x:v>
+      </x:c>
+      <x:c r="C32" s="3" t="str">
+        <x:v>RT-05.21; observación prioritaria 4.</x:v>
+      </x:c>
+      <x:c r="D32" s="3" t="str">
+        <x:v>4.1 catálogo y anexos G–I</x:v>
+      </x:c>
+      <x:c r="E32" s="3" t="str">
+        <x:v>Quince fichas con unidades, fórmulas, ventanas requeridas y conducta ante lentitud/error. Se elimina total agregado que mezclaba unidades y dobles conteos.</x:v>
+      </x:c>
+      <x:c r="F32" s="3" t="str">
+        <x:v>Anexos G, H e I.</x:v>
+      </x:c>
+      <x:c r="G32" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H32" s="3" t="str">
+        <x:v>Catálogo documental ampliado; SLA de terceros y supuestos requieren contrato/medición.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="150" customHeight="1">
+      <x:c r="A33" s="3" t="str">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B33" s="3" t="str">
+        <x:v>Verificar correspondencia completa capítulo 3–lógica–física.</x:v>
+      </x:c>
+      <x:c r="C33" s="3" t="str">
+        <x:v>Aclaraciones capítulo 4; observación 6.</x:v>
+      </x:c>
+      <x:c r="D33" s="3" t="str">
+        <x:v>4.1 relación de vistas</x:v>
+      </x:c>
+      <x:c r="E33" s="3" t="str">
+        <x:v>Anexo N cubre 12 módulos y servicios transversales, señala numeración desactualizada del capítulo 3 y criterio AL-MAP-01.</x:v>
+      </x:c>
+      <x:c r="F33" s="3" t="str">
+        <x:v>Anexo N, tabla de correspondencia.</x:v>
+      </x:c>
+      <x:c r="G33" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H33" s="3" t="str">
+        <x:v>12/12 módulos identificados; no equivale al 100% del inventario integrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="150" customHeight="1">
+      <x:c r="A34" s="3" t="str">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="str">
+        <x:v>Ajustar identificación de entrega y declarar asistencia IA; revisar figuras.</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="str">
+        <x:v>Aclaraciones §§1, 4 y 7.2; observaciones 7 y 8.</x:v>
+      </x:c>
+      <x:c r="D34" s="3" t="str">
+        <x:v>Portada lógica, cierre 4.1 y anexos</x:v>
+      </x:c>
+      <x:c r="E34" s="3" t="str">
+        <x:v>Portada Entrega 2 y declaración de IA con revisión humana aún no realizada. Se preserva la vista de Tomás; quedan diferencias visuales inventariadas.</x:v>
+      </x:c>
+      <x:c r="F34" s="3" t="str">
+        <x:v>main.tex; declaraciones finales; README del 4.1.</x:v>
+      </x:c>
+      <x:c r="G34" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H34" s="3" t="str">
+        <x:v>Formato parcial corregido. Faltan figuras definitivas, revisión humana y capítulo 4 integrado.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
reorganizacion de carpetas y archivos
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R406c256d1ac347b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R4650b984a0c44c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Rd633fa01ff8342f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R3aaca41890c9411c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1380,6 +1380,32 @@
         <x:v>Formato parcial corregido. Faltan figuras definitivas, revisión humana y capítulo 4 integrado.</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="150" customHeight="1">
+      <x:c r="A35" s="3" t="str">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="str">
+        <x:v>Organizar el apartado lógico por archivos editables, siguiendo la estructura modular de 4.2.</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="str">
+        <x:v>Solicitud de Álvaro, 30-09-2026.</x:v>
+      </x:c>
+      <x:c r="D35" s="3" t="str">
+        <x:v>Organización de 4.1 y paquete de distribución</x:v>
+      </x:c>
+      <x:c r="E35" s="3" t="str">
+        <x:v>Se separan 24 fragmentos del cuerpo y 17 de anexos. Se conservan las entradas de compilación y se adapta el exportador.</x:v>
+      </x:c>
+      <x:c r="F35" s="3" t="str">
+        <x:v>Concatenación exacta de fuentes y texto idéntico por página. PDF principal: 60 páginas; anexos: 28.</x:v>
+      </x:c>
+      <x:c r="G35" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H35" s="3" t="str">
+        <x:v>Reorganización implementada sin cambios técnicos ni de arquitectura física. No cierra las brechas de aceptación pendientes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
correcciones, y organizacion de anexos
</commit_message>
<xml_diff>
--- a/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
+++ b/00_trazabilidad_observaciones/tablas/Trazabilidad_Observaciones_Informe1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="Rd633fa01ff8342f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R3aaca41890c9411c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observaciones Informe 1" sheetId="1" r:id="R69a2350842444ecc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R966ddb3e832f4b33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1406,6 +1406,214 @@
         <x:v>Reorganización implementada sin cambios técnicos ni de arquitectura física. No cierra las brechas de aceptación pendientes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="36" ht="150" customHeight="1">
+      <x:c r="A36" s="3" t="str">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="str">
+        <x:v>Catálogo completo y navegación de anexos</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D36" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E36" s="3" t="str">
+        <x:v>22 anexos A–V con enlaces, páginas e identificadores de requisito.</x:v>
+      </x:c>
+      <x:c r="F36" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G36" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H36" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="150" customHeight="1">
+      <x:c r="A37" s="3" t="str">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="str">
+        <x:v>Correspondencia lógica</x:v>
+      </x:c>
+      <x:c r="C37" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D37" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E37" s="3" t="str">
+        <x:v>49 unidades: 12 módulos y 37 capacidades transversales; el cierre integrado exige enlaces físicos exactos.</x:v>
+      </x:c>
+      <x:c r="F37" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G37" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H37" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="150" customHeight="1">
+      <x:c r="A38" s="3" t="str">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B38" s="3" t="str">
+        <x:v>Decisiones verificables</x:v>
+      </x:c>
+      <x:c r="C38" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D38" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E38" s="3" t="str">
+        <x:v>Anexo O con ADR fechados, alternativas, criterios y ensayos; REST API / REQUEST / VPC Link V2 hacia ALB.</x:v>
+      </x:c>
+      <x:c r="F38" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G38" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H38" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="150" customHeight="1">
+      <x:c r="A39" s="3" t="str">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="str">
+        <x:v>Tecnologías y soporte</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D39" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E39" s="3" t="str">
+        <x:v>Anexo P con soporte y actualizaciones durante 56 meses; Terraform propietario y Ansible para hosts.</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G39" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H39" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="150" customHeight="1">
+      <x:c r="A40" s="3" t="str">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B40" s="3" t="str">
+        <x:v>Seguridad lógica</x:v>
+      </x:c>
+      <x:c r="C40" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D40" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E40" s="3" t="str">
+        <x:v>Anexos Q/R: STRIDE por módulo y frontera, controles ISO y evidencia requerida; no declara certificación.</x:v>
+      </x:c>
+      <x:c r="F40" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G40" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H40" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="150" customHeight="1">
+      <x:c r="A41" s="3" t="str">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B41" s="3" t="str">
+        <x:v>Desempeño y evidencia documental</x:v>
+      </x:c>
+      <x:c r="C41" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D41" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E41" s="3" t="str">
+        <x:v>Anexos T/U: percentiles, cargas de 1,5 peak y crecimiento tres veces; POD distinto de acuse tributario.</x:v>
+      </x:c>
+      <x:c r="F41" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G41" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H41" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="150" customHeight="1">
+      <x:c r="A42" s="3" t="str">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B42" s="3" t="str">
+        <x:v>Alcance y condiciones de aceptación</x:v>
+      </x:c>
+      <x:c r="C42" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D42" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E42" s="3" t="str">
+        <x:v>M10/M12 en Etapa 2; Anexo V mantiene decisiones del CLIENTE, ensayos y revisión humana como pendientes.</x:v>
+      </x:c>
+      <x:c r="F42" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G42" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H42" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="150" customHeight="1">
+      <x:c r="A43" s="3" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B43" s="3" t="str">
+        <x:v>Consistencia editorial y figuras</x:v>
+      </x:c>
+      <x:c r="C43" s="3" t="str">
+        <x:v>Plan de mejora aceptado por Álvaro; aclaraciones y bases.</x:v>
+      </x:c>
+      <x:c r="D43" s="3" t="str">
+        <x:v>Arquitectura lógica 4.1</x:v>
+      </x:c>
+      <x:c r="E43" s="3" t="str">
+        <x:v>Referencias técnicas, ADR sin tabla partida y general consolidada del modelo de Tomás; original preservado.</x:v>
+      </x:c>
+      <x:c r="F43" s="3" t="str">
+        <x:v>Fuentes, catálogo de anexos y compilación de distribución.</x:v>
+      </x:c>
+      <x:c r="G43" s="3" t="str">
+        <x:v>LafroX</x:v>
+      </x:c>
+      <x:c r="H43" s="3" t="str">
+        <x:v>Implementación documental; no acredita aprobación del CLIENTE ni ensayos ejecutados.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>